<commit_message>
Promote RW4 pipeline and refresh outputs
</commit_message>
<xml_diff>
--- a/outputs/butter/novus/primary_chain_output.xlsx
+++ b/outputs/butter/novus/primary_chain_output.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PreTests" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelCoefficients" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ResidualDiagnostics" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SeriesUsed" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LagProfile" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelEligibility" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NARDL_Multipliers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VECM_IRF" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PreTests" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ModelCoefficients" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ResidualDiagnostics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SeriesUsed" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="LagProfile" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ModelEligibility" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NARDL_Multipliers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="VECM_IRF" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -518,19 +518,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.08225840900715364</v>
+        <v>0.08225840900720094</v>
       </c>
       <c r="C2" t="n">
         <v>0.01</v>
       </c>
       <c r="D2" t="n">
-        <v>2.681802621264837e-12</v>
+        <v>2.681802621266499e-12</v>
       </c>
       <c r="E2" t="n">
         <v>0.1</v>
       </c>
       <c r="F2" t="n">
-        <v>1.300695796395212e-20</v>
+        <v>1.300695796394998e-20</v>
       </c>
       <c r="G2" t="n">
         <v>0.1</v>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05640422694264773</v>
+        <v>0.05640422694264767</v>
       </c>
       <c r="C3" t="n">
         <v>0.01</v>
@@ -580,7 +580,7 @@
         <v>0.1</v>
       </c>
       <c r="F3" t="n">
-        <v>1.926918418202639e-13</v>
+        <v>1.926918418201579e-13</v>
       </c>
       <c r="G3" t="n">
         <v>0.1</v>
@@ -926,22 +926,22 @@
         <v>218</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.2127764229425361</v>
+        <v>-0.2127764229425364</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2740532058530188</v>
+        <v>0.2740532058530208</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.8083252331134957</v>
+        <v>-0.8083252331134949</v>
       </c>
       <c r="M2" t="n">
-        <v>1.252374581737896e-26</v>
+        <v>1.252374581588286e-26</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7873814868471209</v>
+        <v>0.787381486847105</v>
       </c>
       <c r="O2" t="n">
-        <v>0.2011263550434567</v>
+        <v>0.2011263550434396</v>
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
@@ -1041,10 +1041,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.3043740439991276</v>
+        <v>0.3043740439991278</v>
       </c>
       <c r="F2" t="n">
-        <v>0.5287391650637272</v>
+        <v>0.5287391650637225</v>
       </c>
       <c r="G2" t="n">
         <v>4.220381385301966e-84</v>
@@ -57065,10 +57065,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.5437076425441756</v>
+        <v>-0.5437076425441754</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.3309312196016395</v>
+        <v>-0.330931219601639</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -57081,10 +57081,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.4804346363943778</v>
+        <v>-0.4804346363943776</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.2924196897746271</v>
+        <v>-0.2924196897746266</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -57097,10 +57097,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.4877979195156134</v>
+        <v>-0.4877979195156132</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.2969014002986514</v>
+        <v>-0.2969014002986509</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -57113,10 +57113,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.4869410305889973</v>
+        <v>-0.4869410305889971</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.2963798492381931</v>
+        <v>-0.2963798492381926</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -57129,10 +57129,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.4870407495079181</v>
+        <v>-0.4870407495079179</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.2964405438116616</v>
+        <v>-0.2964405438116611</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -57145,10 +57145,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.4870291448967697</v>
+        <v>-0.4870291448967695</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.2964334805890401</v>
+        <v>-0.2964334805890396</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -57161,10 +57161,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.4870304953626729</v>
+        <v>-0.4870304953626727</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.2964343025589618</v>
+        <v>-0.2964343025589613</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -57177,10 +57177,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.4870303382046146</v>
+        <v>-0.4870303382046144</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.2964342069036797</v>
+        <v>-0.2964342069036792</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -57193,10 +57193,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.487030356493603</v>
+        <v>-0.4870303564936028</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.2964342180353924</v>
+        <v>-0.2964342180353919</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -57209,10 +57209,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.4870303543652547</v>
+        <v>-0.4870303543652544</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.2964342167399592</v>
+        <v>-0.2964342167399587</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -57225,10 +57225,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.4870303546129374</v>
+        <v>-0.4870303546129372</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.2964342168907129</v>
+        <v>-0.2964342168907124</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -57241,10 +57241,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.4870303545841138</v>
+        <v>-0.4870303545841136</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.2964342168731692</v>
+        <v>-0.2964342168731687</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -57257,10 +57257,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.4870303545874681</v>
+        <v>-0.4870303545874679</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.2964342168752108</v>
+        <v>-0.2964342168752103</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -57273,10 +57273,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>-0.4870303545870777</v>
+        <v>-0.4870303545870775</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.2964342168749732</v>
+        <v>-0.2964342168749727</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -57289,10 +57289,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.4870303545871231</v>
+        <v>-0.487030354587123</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.2964342168750009</v>
+        <v>-0.2964342168750004</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -57305,10 +57305,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.4870303545871179</v>
+        <v>-0.4870303545871176</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.2964342168749977</v>
+        <v>-0.2964342168749972</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -57321,10 +57321,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.4870303545871185</v>
+        <v>-0.4870303545871183</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.296434216874998</v>
+        <v>-0.2964342168749975</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -57337,10 +57337,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.4870303545871184</v>
+        <v>-0.4870303545871182</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.296434216874998</v>
+        <v>-0.2964342168749975</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -57353,10 +57353,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.4870303545871184</v>
+        <v>-0.4870303545871182</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.296434216874998</v>
+        <v>-0.2964342168749975</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -57369,10 +57369,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>-0.4870303545871184</v>
+        <v>-0.4870303545871182</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.296434216874998</v>
+        <v>-0.2964342168749975</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -57385,10 +57385,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>-0.4870303545871184</v>
+        <v>-0.4870303545871182</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.296434216874998</v>
+        <v>-0.2964342168749975</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>

</xml_diff>